<commit_message>
Changed Device Configuration Pak-Device-2
</commit_message>
<xml_diff>
--- a/Embedded Dev/Firmware Development/_Documents/Devices-Database.xlsx
+++ b/Embedded Dev/Firmware Development/_Documents/Devices-Database.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24411"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6C665B4-5633-47C1-8BA0-018C926D48C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -111,7 +112,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -276,6 +277,142 @@
   </cellStyles>
   <dxfs count="9">
     <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <strike val="0"/>
@@ -297,142 +434,6 @@
         </right>
         <top/>
         <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
       </border>
     </dxf>
   </dxfs>
@@ -449,14 +450,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:E11" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="7" tableBorderDxfId="8" totalsRowBorderDxfId="6">
-  <autoFilter ref="A1:E11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:E11" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="7" tableBorderDxfId="6" totalsRowBorderDxfId="5">
+  <autoFilter ref="A1:E11" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" name="S.No" dataDxfId="5"/>
-    <tableColumn id="2" name="Device-ID" dataDxfId="4"/>
-    <tableColumn id="3" name="Device Name" dataDxfId="3"/>
-    <tableColumn id="4" name="Remarks" dataDxfId="2"/>
-    <tableColumn id="5" name="Status" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="S.No" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Device-ID" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Device Name" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Remarks" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Status" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -724,18 +725,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.28515625" customWidth="1"/>
-    <col min="3" max="3" width="16.5703125" customWidth="1"/>
-    <col min="4" max="4" width="19.5703125" customWidth="1"/>
+    <col min="1" max="1" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.33203125" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" customWidth="1"/>
+    <col min="4" max="4" width="19.5546875" customWidth="1"/>
     <col min="5" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -752,7 +753,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -769,7 +770,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -786,7 +787,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -803,7 +804,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -820,7 +821,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -837,7 +838,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -854,7 +855,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -871,7 +872,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -888,7 +889,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -902,10 +903,10 @@
         <v>21</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>10</v>
       </c>

</xml_diff>